<commit_message>
docs: melhoria de documentação, testes e configurações
- Dividir GUIA.md em 7 arquivos menores (GUIA-01 a GUIA-07) para facilitar navegação
- Adicionar CODE_OF_CONDUCT.md (Contributor Covenant v2.1)
- Melhorar CONTRIBUTING.md com exemplos de commits com scope e regras de atomicidade
- Fix cobertura: excluir ports e type-only files do coverage threshold (vitest.config.ts)
- Fix ESLint: ignorar scripts/**/*.mjs no eslint.config.js
- Remover dependências duplicadas (tsx do infrastructure, typescript do frontend)
- Adicionar image-preprocessor para pré-processamento de imagens OCR
- Atualizar exemplos de output com novos formatos
- Atualizar configurações OCR e testes de integração
</commit_message>
<xml_diff>
--- a/exemplos/output/time-card-02.xlsx
+++ b/exemplos/output/time-card-02.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="225">
   <si>
     <t>Data</t>
   </si>
@@ -118,10 +118,7 @@
     <t>25/05/2010</t>
   </si>
   <si>
-    <t>12:54</t>
-  </si>
-  <si>
-    <t>13:56</t>
+    <t>08:57</t>
   </si>
   <si>
     <t>26/05/2010</t>
@@ -139,10 +136,10 @@
     <t>28/05/2010</t>
   </si>
   <si>
-    <t>12:03</t>
-  </si>
-  <si>
-    <t>13:04</t>
+    <t>08:00</t>
+  </si>
+  <si>
+    <t>17:01</t>
   </si>
   <si>
     <t>29/05/2010</t>
@@ -157,24 +154,63 @@
     <t>15:15</t>
   </si>
   <si>
+    <t>01/06/2010</t>
+  </si>
+  <si>
+    <t>10:36</t>
+  </si>
+  <si>
+    <t>16:52</t>
+  </si>
+  <si>
     <t>02/06/2010</t>
   </si>
   <si>
-    <t>14:00</t>
-  </si>
-  <si>
-    <t>14:15</t>
+    <t>10:43</t>
+  </si>
+  <si>
+    <t>16:58</t>
   </si>
   <si>
     <t>03/06/2010</t>
   </si>
   <si>
+    <t>04/06/2010</t>
+  </si>
+  <si>
+    <t>10:41</t>
+  </si>
+  <si>
+    <t>16:56</t>
+  </si>
+  <si>
     <t>05/06/2010</t>
   </si>
   <si>
     <t>06/06/2010</t>
   </si>
   <si>
+    <t>07/06/2010</t>
+  </si>
+  <si>
+    <t>08/06/2010</t>
+  </si>
+  <si>
+    <t>10:46</t>
+  </si>
+  <si>
+    <t>17:00</t>
+  </si>
+  <si>
+    <t>09/06/2010</t>
+  </si>
+  <si>
+    <t>10:39</t>
+  </si>
+  <si>
+    <t>16:55</t>
+  </si>
+  <si>
     <t>10/06/2010</t>
   </si>
   <si>
@@ -190,19 +226,13 @@
     <t>14/06/2010</t>
   </si>
   <si>
-    <t>10:36</t>
-  </si>
-  <si>
-    <t>16:52</t>
-  </si>
-  <si>
     <t>15/06/2010</t>
   </si>
   <si>
-    <t>11:01</t>
-  </si>
-  <si>
-    <t>11:16</t>
+    <t>08:01</t>
+  </si>
+  <si>
+    <t>14:16</t>
   </si>
   <si>
     <t>16/06/2010</t>
@@ -217,9 +247,6 @@
     <t>10:45</t>
   </si>
   <si>
-    <t>17:01</t>
-  </si>
-  <si>
     <t>18/06/2010</t>
   </si>
   <si>
@@ -238,30 +265,18 @@
     <t>21/06/2010</t>
   </si>
   <si>
-    <t>10:39</t>
-  </si>
-  <si>
     <t>16:54</t>
   </si>
   <si>
     <t>22/06/2010</t>
   </si>
   <si>
-    <t>10:41</t>
-  </si>
-  <si>
-    <t>16:56</t>
-  </si>
-  <si>
     <t>23/06/2010</t>
   </si>
   <si>
     <t>10:40</t>
   </si>
   <si>
-    <t>16:55</t>
-  </si>
-  <si>
     <t>24/06/2010</t>
   </si>
   <si>
@@ -283,10 +298,10 @@
     <t>28/06/2010</t>
   </si>
   <si>
-    <t>11:46</t>
-  </si>
-  <si>
-    <t>12:01</t>
+    <t>08:46</t>
+  </si>
+  <si>
+    <t>15:00</t>
   </si>
   <si>
     <t>29/06/2010</t>
@@ -319,6 +334,39 @@
     <t>04/07/2010</t>
   </si>
   <si>
+    <t>05/07/2010</t>
+  </si>
+  <si>
+    <t>09:58</t>
+  </si>
+  <si>
+    <t>16:14</t>
+  </si>
+  <si>
+    <t>06/07/2010</t>
+  </si>
+  <si>
+    <t>09:54</t>
+  </si>
+  <si>
+    <t>16:10</t>
+  </si>
+  <si>
+    <t>07/07/2010</t>
+  </si>
+  <si>
+    <t>09:53</t>
+  </si>
+  <si>
+    <t>16:08</t>
+  </si>
+  <si>
+    <t>08/07/2010</t>
+  </si>
+  <si>
+    <t>09:52</t>
+  </si>
+  <si>
     <t>09/07/2010</t>
   </si>
   <si>
@@ -379,12 +427,6 @@
     <t>22/07/2010</t>
   </si>
   <si>
-    <t>09:53</t>
-  </si>
-  <si>
-    <t>16:08</t>
-  </si>
-  <si>
     <t>23/07/2010</t>
   </si>
   <si>
@@ -397,9 +439,6 @@
     <t>26/07/2010</t>
   </si>
   <si>
-    <t>09:52</t>
-  </si>
-  <si>
     <t>27/07/2010</t>
   </si>
   <si>
@@ -430,6 +469,30 @@
     <t>15:59</t>
   </si>
   <si>
+    <t>03/08/2010</t>
+  </si>
+  <si>
+    <t>08:52</t>
+  </si>
+  <si>
+    <t>16:16</t>
+  </si>
+  <si>
+    <t>04/08/2010</t>
+  </si>
+  <si>
+    <t>08:48</t>
+  </si>
+  <si>
+    <t>05/08/2010</t>
+  </si>
+  <si>
+    <t>08:51</t>
+  </si>
+  <si>
+    <t>15:51</t>
+  </si>
+  <si>
     <t>06/08/2010</t>
   </si>
   <si>
@@ -439,13 +502,16 @@
     <t>08/08/2010</t>
   </si>
   <si>
+    <t>09/08/2010</t>
+  </si>
+  <si>
+    <t>16:04</t>
+  </si>
+  <si>
     <t>10/08/2010</t>
   </si>
   <si>
-    <t>11:51</t>
-  </si>
-  <si>
-    <t>12:06</t>
+    <t>15:49</t>
   </si>
   <si>
     <t>11/08/2010</t>
@@ -457,6 +523,9 @@
     <t>13/08/2010</t>
   </si>
   <si>
+    <t>15:50</t>
+  </si>
+  <si>
     <t>14/08/2010</t>
   </si>
   <si>
@@ -469,18 +538,9 @@
     <t>17/08/2010</t>
   </si>
   <si>
-    <t>13:00</t>
-  </si>
-  <si>
-    <t>13:15</t>
-  </si>
-  <si>
     <t>18/08/2010</t>
   </si>
   <si>
-    <t>16:10</t>
-  </si>
-  <si>
     <t>19/08/2010</t>
   </si>
   <si>
@@ -526,33 +586,45 @@
     <t>02/09/2010</t>
   </si>
   <si>
+    <t>03/09/2010</t>
+  </si>
+  <si>
+    <t>15:42</t>
+  </si>
+  <si>
     <t>04/09/2010</t>
   </si>
   <si>
     <t>05/09/2010</t>
   </si>
   <si>
+    <t>06/09/2010</t>
+  </si>
+  <si>
+    <t>08:55</t>
+  </si>
+  <si>
+    <t>15:47</t>
+  </si>
+  <si>
     <t>07/09/2010</t>
   </si>
   <si>
+    <t>08/09/2010</t>
+  </si>
+  <si>
+    <t>15:53</t>
+  </si>
+  <si>
     <t>09/09/2010</t>
   </si>
   <si>
-    <t>11:50</t>
-  </si>
-  <si>
-    <t>12:05</t>
+    <t>08:50</t>
   </si>
   <si>
     <t>10/09/2010</t>
   </si>
   <si>
-    <t>11:55</t>
-  </si>
-  <si>
-    <t>12:10</t>
-  </si>
-  <si>
     <t>11/09/2010</t>
   </si>
   <si>
@@ -593,9 +665,6 @@
   </si>
   <si>
     <t>24/09/2010</t>
-  </si>
-  <si>
-    <t>09:54</t>
   </si>
   <si>
     <t>16:09</t>
@@ -636,7 +705,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -648,24 +717,10 @@
         <fgColor rgb="FF173772"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8D7DA"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FFDC3545"/>
-      </left>
       <right/>
       <top/>
       <bottom/>
@@ -675,10 +730,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1018,7 +1072,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C154"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="18" customWidth="1"/>
@@ -1307,23 +1361,23 @@
         <v>35</v>
       </c>
       <c r="C26" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>36</v>
+      </c>
+      <c r="B27" t="s">
         <v>37</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>38</v>
-      </c>
-      <c r="C27" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B28" t="s">
         <v>24</v>
@@ -1334,18 +1388,18 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" t="s">
         <v>41</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>42</v>
-      </c>
-      <c r="C29" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B30" t="s">
         <v>4</v>
@@ -1356,7 +1410,7 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B31" t="s">
         <v>4</v>
@@ -1367,145 +1421,145 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B32" t="s">
         <v>24</v>
       </c>
       <c r="C32" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
+      <c r="B33" t="s">
         <v>48</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="C33" t="s">
         <v>49</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>50</v>
+      </c>
+      <c r="B34" t="s">
         <v>51</v>
       </c>
-      <c r="B34" t="s">
-        <v>4</v>
-      </c>
       <c r="C34" t="s">
-        <v>4</v>
+        <v>52</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C35" s="2" t="s">
+      <c r="A35" t="s">
+        <v>53</v>
+      </c>
+      <c r="B35" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B36" t="s">
-        <v>4</v>
+        <v>55</v>
       </c>
       <c r="C36" t="s">
-        <v>4</v>
+        <v>56</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>50</v>
+      <c r="A37" t="s">
+        <v>57</v>
+      </c>
+      <c r="B37" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B38" t="s">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="C38" t="s">
-        <v>50</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>59</v>
+      </c>
+      <c r="B39" t="s">
+        <v>55</v>
+      </c>
+      <c r="C39" t="s">
         <v>56</v>
-      </c>
-      <c r="B39" t="s">
-        <v>4</v>
-      </c>
-      <c r="C39" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B40" t="s">
-        <v>4</v>
+        <v>61</v>
       </c>
       <c r="C40" t="s">
-        <v>4</v>
+        <v>62</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B41" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C41" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B42" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C42" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B43" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="C43" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B44" t="s">
-        <v>67</v>
+        <v>4</v>
       </c>
       <c r="C44" t="s">
-        <v>68</v>
+        <v>4</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -1513,32 +1567,32 @@
         <v>69</v>
       </c>
       <c r="B45" t="s">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="C45" t="s">
-        <v>71</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B46" t="s">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="C46" t="s">
-        <v>4</v>
+        <v>49</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>71</v>
+      </c>
+      <c r="B47" t="s">
+        <v>72</v>
+      </c>
+      <c r="C47" t="s">
         <v>73</v>
-      </c>
-      <c r="B47" t="s">
-        <v>4</v>
-      </c>
-      <c r="C47" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -1546,186 +1600,186 @@
         <v>74</v>
       </c>
       <c r="B48" t="s">
+        <v>48</v>
+      </c>
+      <c r="C48" t="s">
         <v>75</v>
-      </c>
-      <c r="C48" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>76</v>
+      </c>
+      <c r="B49" t="s">
         <v>77</v>
       </c>
-      <c r="B49" t="s">
-        <v>78</v>
-      </c>
       <c r="C49" t="s">
-        <v>79</v>
+        <v>42</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>78</v>
+      </c>
+      <c r="B50" t="s">
+        <v>79</v>
+      </c>
+      <c r="C50" t="s">
         <v>80</v>
-      </c>
-      <c r="B50" t="s">
-        <v>81</v>
-      </c>
-      <c r="C50" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B51" t="s">
-        <v>75</v>
+        <v>4</v>
       </c>
       <c r="C51" t="s">
-        <v>76</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B52" t="s">
-        <v>85</v>
+        <v>4</v>
       </c>
       <c r="C52" t="s">
-        <v>86</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B53" t="s">
-        <v>4</v>
+        <v>64</v>
       </c>
       <c r="C53" t="s">
-        <v>4</v>
+        <v>84</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B54" t="s">
-        <v>4</v>
+        <v>55</v>
       </c>
       <c r="C54" t="s">
-        <v>4</v>
+        <v>56</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B55" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C55" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B56" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="C56" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B57" t="s">
-        <v>49</v>
+        <v>90</v>
       </c>
       <c r="C57" t="s">
-        <v>50</v>
+        <v>91</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B58" t="s">
-        <v>95</v>
+        <v>4</v>
       </c>
       <c r="C58" t="s">
-        <v>96</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B59" t="s">
-        <v>98</v>
+        <v>4</v>
       </c>
       <c r="C59" t="s">
-        <v>99</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B60" t="s">
-        <v>4</v>
+        <v>95</v>
       </c>
       <c r="C60" t="s">
-        <v>4</v>
+        <v>96</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B61" t="s">
-        <v>4</v>
+        <v>64</v>
       </c>
       <c r="C61" t="s">
-        <v>4</v>
+        <v>84</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>4</v>
+      <c r="A62" t="s">
+        <v>98</v>
+      </c>
+      <c r="B62" t="s">
+        <v>87</v>
+      </c>
+      <c r="C62" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B63" t="s">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="C63" t="s">
-        <v>4</v>
+        <v>101</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>102</v>
+      </c>
+      <c r="B64" t="s">
+        <v>103</v>
+      </c>
+      <c r="C64" t="s">
         <v>104</v>
-      </c>
-      <c r="B64" t="s">
-        <v>4</v>
-      </c>
-      <c r="C64" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
@@ -1733,32 +1787,32 @@
         <v>105</v>
       </c>
       <c r="B65" t="s">
-        <v>106</v>
+        <v>4</v>
       </c>
       <c r="C65" t="s">
-        <v>107</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B66" t="s">
-        <v>106</v>
+        <v>4</v>
       </c>
       <c r="C66" t="s">
-        <v>107</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>107</v>
+      </c>
+      <c r="B67" t="s">
+        <v>108</v>
+      </c>
+      <c r="C67" t="s">
         <v>109</v>
-      </c>
-      <c r="B67" t="s">
-        <v>106</v>
-      </c>
-      <c r="C67" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
@@ -1766,37 +1820,37 @@
         <v>110</v>
       </c>
       <c r="B68" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C68" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B69" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C69" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B70" t="s">
-        <v>4</v>
+        <v>117</v>
       </c>
       <c r="C70" t="s">
-        <v>4</v>
+        <v>101</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B71" t="s">
         <v>4</v>
@@ -1807,40 +1861,40 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B72" t="s">
-        <v>95</v>
+        <v>4</v>
       </c>
       <c r="C72" t="s">
-        <v>107</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="B73" t="s">
-        <v>116</v>
+        <v>4</v>
       </c>
       <c r="C73" t="s">
-        <v>117</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B74" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C74" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B75" t="s">
         <v>122</v>
@@ -1851,10 +1905,10 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B76" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="C76" t="s">
         <v>123</v>
@@ -1862,35 +1916,35 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B77" t="s">
-        <v>4</v>
+        <v>122</v>
       </c>
       <c r="C77" t="s">
-        <v>4</v>
+        <v>123</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B78" t="s">
-        <v>4</v>
+        <v>122</v>
       </c>
       <c r="C78" t="s">
-        <v>4</v>
+        <v>123</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B79" t="s">
-        <v>128</v>
+        <v>4</v>
       </c>
       <c r="C79" t="s">
-        <v>96</v>
+        <v>4</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
@@ -1898,10 +1952,10 @@
         <v>129</v>
       </c>
       <c r="B80" t="s">
-        <v>106</v>
+        <v>4</v>
       </c>
       <c r="C80" t="s">
-        <v>107</v>
+        <v>4</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
@@ -1909,108 +1963,108 @@
         <v>130</v>
       </c>
       <c r="B81" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C81" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>131</v>
+      </c>
+      <c r="B82" t="s">
         <v>132</v>
       </c>
-      <c r="B82" t="s">
-        <v>95</v>
-      </c>
       <c r="C82" t="s">
-        <v>107</v>
+        <v>133</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B83" t="s">
-        <v>106</v>
+        <v>135</v>
       </c>
       <c r="C83" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B84" t="s">
-        <v>4</v>
+        <v>114</v>
       </c>
       <c r="C84" t="s">
-        <v>4</v>
+        <v>115</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B85" t="s">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="C85" t="s">
-        <v>4</v>
+        <v>115</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B86" t="s">
-        <v>137</v>
+        <v>4</v>
       </c>
       <c r="C86" t="s">
-        <v>138</v>
+        <v>4</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A87" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C87" s="2" t="s">
+      <c r="A87" t="s">
+        <v>140</v>
+      </c>
+      <c r="B87" t="s">
+        <v>4</v>
+      </c>
+      <c r="C87" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B88" t="s">
-        <v>4</v>
+        <v>117</v>
       </c>
       <c r="C88" t="s">
-        <v>4</v>
+        <v>101</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B89" t="s">
-        <v>4</v>
+        <v>122</v>
       </c>
       <c r="C89" t="s">
-        <v>4</v>
+        <v>123</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A90" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="B90" s="2" t="s">
+      <c r="A90" t="s">
         <v>143</v>
       </c>
-      <c r="C90" s="2" t="s">
+      <c r="B90" t="s">
+        <v>122</v>
+      </c>
+      <c r="C90" t="s">
         <v>144</v>
       </c>
     </row>
@@ -2019,10 +2073,10 @@
         <v>145</v>
       </c>
       <c r="B91" t="s">
-        <v>143</v>
+        <v>100</v>
       </c>
       <c r="C91" t="s">
-        <v>144</v>
+        <v>123</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
@@ -2030,7 +2084,7 @@
         <v>146</v>
       </c>
       <c r="B92" t="s">
-        <v>143</v>
+        <v>122</v>
       </c>
       <c r="C92" t="s">
         <v>144</v>
@@ -2041,10 +2095,10 @@
         <v>147</v>
       </c>
       <c r="B93" t="s">
-        <v>143</v>
+        <v>4</v>
       </c>
       <c r="C93" t="s">
-        <v>144</v>
+        <v>4</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
@@ -2063,70 +2117,70 @@
         <v>149</v>
       </c>
       <c r="B95" t="s">
-        <v>4</v>
+        <v>150</v>
       </c>
       <c r="C95" t="s">
-        <v>4</v>
+        <v>151</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B96" t="s">
-        <v>106</v>
+        <v>153</v>
       </c>
       <c r="C96" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B97" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C97" t="s">
-        <v>153</v>
+        <v>133</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B98" t="s">
-        <v>116</v>
+        <v>158</v>
       </c>
       <c r="C98" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B99" t="s">
-        <v>128</v>
+        <v>4</v>
       </c>
       <c r="C99" t="s">
-        <v>96</v>
+        <v>4</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B100" t="s">
-        <v>128</v>
+        <v>4</v>
       </c>
       <c r="C100" t="s">
-        <v>96</v>
+        <v>4</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B101" t="s">
         <v>4</v>
@@ -2137,73 +2191,73 @@
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B102" t="s">
-        <v>4</v>
+        <v>158</v>
       </c>
       <c r="C102" t="s">
-        <v>4</v>
+        <v>164</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B103" t="s">
-        <v>116</v>
+        <v>158</v>
       </c>
       <c r="C103" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B104" t="s">
-        <v>116</v>
+        <v>158</v>
       </c>
       <c r="C104" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B105" t="s">
-        <v>116</v>
+        <v>158</v>
       </c>
       <c r="C105" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B106" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="C106" t="s">
-        <v>107</v>
+        <v>170</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B107" t="s">
-        <v>106</v>
+        <v>4</v>
       </c>
       <c r="C107" t="s">
-        <v>131</v>
+        <v>4</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="B108" t="s">
         <v>4</v>
@@ -2214,73 +2268,73 @@
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="B109" t="s">
-        <v>4</v>
+        <v>122</v>
       </c>
       <c r="C109" t="s">
-        <v>4</v>
+        <v>144</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="B110" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C110" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="B111" t="s">
-        <v>106</v>
+        <v>132</v>
       </c>
       <c r="C111" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="B112" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="C112" t="s">
-        <v>131</v>
+        <v>101</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="B113" t="s">
-        <v>95</v>
+        <v>117</v>
       </c>
       <c r="C113" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A114" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="B114" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C114" s="2" t="s">
+      <c r="A114" t="s">
+        <v>178</v>
+      </c>
+      <c r="B114" t="s">
+        <v>4</v>
+      </c>
+      <c r="C114" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="B115" t="s">
         <v>4</v>
@@ -2290,256 +2344,432 @@
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A116" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="B116" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C116" s="2" t="s">
-        <v>4</v>
+      <c r="A116" t="s">
+        <v>180</v>
+      </c>
+      <c r="B116" t="s">
+        <v>132</v>
+      </c>
+      <c r="C116" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A117" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="B117" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="C117" s="2" t="s">
-        <v>176</v>
+      <c r="A117" t="s">
+        <v>181</v>
+      </c>
+      <c r="B117" t="s">
+        <v>132</v>
+      </c>
+      <c r="C117" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B118" t="s">
-        <v>178</v>
+        <v>132</v>
       </c>
       <c r="C118" t="s">
-        <v>179</v>
+        <v>112</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B119" t="s">
-        <v>4</v>
+        <v>122</v>
       </c>
       <c r="C119" t="s">
-        <v>4</v>
+        <v>123</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B120" t="s">
-        <v>4</v>
+        <v>122</v>
       </c>
       <c r="C120" t="s">
-        <v>4</v>
+        <v>144</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B121" t="s">
-        <v>106</v>
+        <v>4</v>
       </c>
       <c r="C121" t="s">
-        <v>131</v>
+        <v>4</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B122" t="s">
-        <v>95</v>
+        <v>4</v>
       </c>
       <c r="C122" t="s">
-        <v>107</v>
+        <v>4</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B123" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="C123" t="s">
-        <v>155</v>
+        <v>123</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B124" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="C124" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B125" t="s">
         <v>122</v>
       </c>
       <c r="C125" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B126" t="s">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="C126" t="s">
-        <v>4</v>
+        <v>123</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B127" t="s">
-        <v>4</v>
+        <v>153</v>
       </c>
       <c r="C127" t="s">
-        <v>4</v>
+        <v>192</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B128" t="s">
-        <v>128</v>
+        <v>4</v>
       </c>
       <c r="C128" t="s">
-        <v>96</v>
+        <v>4</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B129" t="s">
-        <v>95</v>
+        <v>4</v>
       </c>
       <c r="C129" t="s">
-        <v>107</v>
+        <v>4</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B130" t="s">
-        <v>128</v>
+        <v>196</v>
       </c>
       <c r="C130" t="s">
-        <v>96</v>
+        <v>197</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B131" t="s">
-        <v>128</v>
+        <v>4</v>
       </c>
       <c r="C131" t="s">
-        <v>96</v>
+        <v>4</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="B132" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C132" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="B133" t="s">
-        <v>4</v>
+        <v>202</v>
       </c>
       <c r="C133" t="s">
-        <v>4</v>
+        <v>197</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="B134" t="s">
-        <v>4</v>
+        <v>196</v>
       </c>
       <c r="C134" t="s">
-        <v>4</v>
+        <v>159</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="B135" t="s">
-        <v>106</v>
+        <v>4</v>
       </c>
       <c r="C135" t="s">
-        <v>131</v>
+        <v>4</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="B136" t="s">
-        <v>106</v>
+        <v>4</v>
       </c>
       <c r="C136" t="s">
-        <v>131</v>
+        <v>4</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="B137" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="C137" t="s">
-        <v>117</v>
+        <v>144</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B138" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C138" t="s">
-        <v>131</v>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>208</v>
+      </c>
+      <c r="B139" t="s">
+        <v>132</v>
+      </c>
+      <c r="C139" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>209</v>
+      </c>
+      <c r="B140" t="s">
+        <v>122</v>
+      </c>
+      <c r="C140" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>210</v>
+      </c>
+      <c r="B141" t="s">
+        <v>114</v>
+      </c>
+      <c r="C141" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>211</v>
+      </c>
+      <c r="B142" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>212</v>
+      </c>
+      <c r="B143" t="s">
+        <v>4</v>
+      </c>
+      <c r="C143" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>213</v>
+      </c>
+      <c r="B144" t="s">
+        <v>117</v>
+      </c>
+      <c r="C144" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>214</v>
+      </c>
+      <c r="B145" t="s">
+        <v>100</v>
+      </c>
+      <c r="C145" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>215</v>
+      </c>
+      <c r="B146" t="s">
+        <v>117</v>
+      </c>
+      <c r="C146" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>216</v>
+      </c>
+      <c r="B147" t="s">
+        <v>117</v>
+      </c>
+      <c r="C147" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>217</v>
+      </c>
+      <c r="B148" t="s">
+        <v>111</v>
+      </c>
+      <c r="C148" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>219</v>
+      </c>
+      <c r="B149" t="s">
+        <v>4</v>
+      </c>
+      <c r="C149" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>220</v>
+      </c>
+      <c r="B150" t="s">
+        <v>4</v>
+      </c>
+      <c r="C150" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>221</v>
+      </c>
+      <c r="B151" t="s">
+        <v>122</v>
+      </c>
+      <c r="C151" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>222</v>
+      </c>
+      <c r="B152" t="s">
+        <v>122</v>
+      </c>
+      <c r="C152" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>223</v>
+      </c>
+      <c r="B153" t="s">
+        <v>132</v>
+      </c>
+      <c r="C153" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>224</v>
+      </c>
+      <c r="B154" t="s">
+        <v>122</v>
+      </c>
+      <c r="C154" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>